<commit_message>
elec updates - BRPSDbS, GBCGpUNR, and CSC
</commit_message>
<xml_diff>
--- a/InputData/elec/CSC/Capacity Supply Curve.xlsx
+++ b/InputData/elec/CSC/Capacity Supply Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\CSC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\elec\CSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55974A76-ACCE-4EEE-8FAE-8F68F7567405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FF53E0-7987-44DF-AA05-C83B053F824F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
+    <workbookView xWindow="2604" yWindow="960" windowWidth="18660" windowHeight="12228" activeTab="1" xr2:uid="{F87DB1D1-DC21-4EA7-B1DF-998EE56837F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -609,307 +609,307 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="101"/>
                 <c:pt idx="0">
-                  <c:v>2.9387164590499728E-6</c:v>
+                  <c:v>1.8084408978769062E-6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.3508987656584158E-5</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.9336018158404631E-5</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.8802429327882398E-4</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.6713369702505162E-4</c:v>
+                  <c:v>2.2592842893849331E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.3414614007045462E-4</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.006422790718059E-3</c:v>
+                  <c:v>6.1933710198034406E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.5011520593627675E-3</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.1352885583158314E-3</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.9254833434584626E-3</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.8880058412656712E-3</c:v>
+                  <c:v>2.3926189792404132E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.0386579732422526E-3</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>6.3926811083940913E-3</c:v>
+                  <c:v>3.9339576051655948E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>7.9646566013662247E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>9.7684008073131972E-3</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.1816855602081967E-2</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.4121975575197189E-2</c:v>
+                  <c:v>8.6904465078136549E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.6694613200417676E-2</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.9544403420951564E-2</c:v>
+                  <c:v>1.2027325182124038E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.267964921017894E-2</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.6107209780122643E-2</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2.9832393204970647E-2</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>3.3858855301670994E-2</c:v>
+                  <c:v>2.0836218647182148E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.8188506660006477E-2</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>4.2821429736777793E-2</c:v>
+                  <c:v>2.6351649068786332E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>4.7755807919210802E-2</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>5.2987868418287974E-2</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.8511840770746393E-2</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>6.4319932607017835E-2</c:v>
+                  <c:v>3.9581496988934053E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>7.040232418023408E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.6747182948336296E-2</c:v>
+                  <c:v>4.7229035660514646E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>8.3340699258080464E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>9.0167143898212704E-2</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>9.7208947972360321E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>0.10444680519450757</c:v>
+                  <c:v>6.4274957042773889E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.11185979633676199</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.11942553516706651</c:v>
+                  <c:v>7.3492637025887084E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.12712033481123883</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.13491939306780171</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.14279699480482452</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.15072672918526989</c:v>
+                  <c:v>9.2754910267858384E-2</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>0.15868171911122922</c:v>
+                  <c:v>9.7650288683833367E-2</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>0.16663485995800573</c:v>
+                  <c:v>0.10254452920492661</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>0.17455906439599175</c:v>
+                  <c:v>0.10742096270522571</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>0.18242750988073522</c:v>
+                  <c:v>0.11226308300352937</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>0.19021388523755758</c:v>
+                  <c:v>0.11705469860772776</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>0.19789263268329291</c:v>
+                  <c:v>0.12178008165125719</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>0.20543918161928124</c:v>
+                  <c:v>0.12642411176571153</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>0.21283017059990736</c:v>
+                  <c:v>0.13097241267686607</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>0.22004365403087262</c:v>
+                  <c:v>0.13541147940361392</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>0.22705929037995962</c:v>
+                  <c:v>0.13972879407997515</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>0.23385850898689628</c:v>
+                  <c:v>0.1439129286073208</c:v>
                 </c:pt>
                 <c:pt idx="52">
-                  <c:v>0.24042465293238419</c:v>
+                  <c:v>0.14795363257377489</c:v>
                 </c:pt>
                 <c:pt idx="53">
-                  <c:v>0.2467430958615193</c:v>
+                  <c:v>0.15184190514555035</c:v>
                 </c:pt>
                 <c:pt idx="54">
-                  <c:v>0.25280133114377951</c:v>
+                  <c:v>0.15557004993463353</c:v>
                 </c:pt>
                 <c:pt idx="55">
-                  <c:v>0.2585890322787715</c:v>
+                  <c:v>0.1591317121715517</c:v>
                 </c:pt>
                 <c:pt idx="56">
-                  <c:v>0.26409808401086282</c:v>
+                  <c:v>0.16252189785283866</c:v>
                 </c:pt>
                 <c:pt idx="57">
-                  <c:v>0.26932258418246974</c:v>
+                  <c:v>0.16573697488151984</c:v>
                 </c:pt>
                 <c:pt idx="58">
-                  <c:v>0.27425881692032672</c:v>
+                  <c:v>0.16877465656635493</c:v>
                 </c:pt>
                 <c:pt idx="59">
-                  <c:v>0.2789051982966137</c:v>
+                  <c:v>0.17163396818253152</c:v>
                 </c:pt>
                 <c:pt idx="60">
-                  <c:v>0.28326219612285092</c:v>
+                  <c:v>0.17431519761406211</c:v>
                 </c:pt>
                 <c:pt idx="61">
-                  <c:v>0.2873322260053523</c:v>
+                  <c:v>0.17681983138790913</c:v>
                 </c:pt>
                 <c:pt idx="62">
-                  <c:v>0.29111952620450759</c:v>
+                  <c:v>0.17915047766431236</c:v>
                 </c:pt>
                 <c:pt idx="63">
-                  <c:v>0.29463001418577178</c:v>
+                  <c:v>0.18131077796047496</c:v>
                 </c:pt>
                 <c:pt idx="64">
-                  <c:v>0.29787112801967686</c:v>
+                  <c:v>0.18330530955057037</c:v>
                 </c:pt>
                 <c:pt idx="65">
-                  <c:v>0.30085165597558955</c:v>
+                  <c:v>0.18513948060036278</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>0.30358155775609158</c:v>
+                  <c:v>0.18681942015759484</c:v>
                 </c:pt>
                 <c:pt idx="67">
-                  <c:v>0.30607178083525383</c:v>
+                  <c:v>0.18835186512938695</c:v>
                 </c:pt>
                 <c:pt idx="68">
-                  <c:v>0.30833407529690587</c:v>
+                  <c:v>0.18974404633655748</c:v>
                 </c:pt>
                 <c:pt idx="69">
-                  <c:v>0.31038081042304033</c:v>
+                  <c:v>0.19100357564494788</c:v>
                 </c:pt>
                 <c:pt idx="70">
-                  <c:v>0.31222479606484704</c:v>
+                  <c:v>0.19213833603990588</c:v>
                 </c:pt>
                 <c:pt idx="71">
-                  <c:v>0.31387911154870857</c:v>
+                  <c:v>0.1931563763376668</c:v>
                 </c:pt>
                 <c:pt idx="72">
-                  <c:v>0.31535694453758484</c:v>
+                  <c:v>0.19406581202312914</c:v>
                 </c:pt>
                 <c:pt idx="73">
-                  <c:v>0.31667144189658553</c:v>
+                  <c:v>0.19487473347482187</c:v>
                 </c:pt>
                 <c:pt idx="74">
-                  <c:v>0.3178355742128724</c:v>
+                  <c:v>0.19559112259253686</c:v>
                 </c:pt>
                 <c:pt idx="75">
-                  <c:v>0.31886201520731511</c:v>
+                  <c:v>0.19622277858911699</c:v>
                 </c:pt>
                 <c:pt idx="76">
-                  <c:v>0.31976303686122226</c:v>
+                  <c:v>0.19677725345305985</c:v>
                 </c:pt>
                 <c:pt idx="77">
-                  <c:v>0.32055042067798994</c:v>
+                  <c:v>0.1972617973403015</c:v>
                 </c:pt>
                 <c:pt idx="78">
-                  <c:v>0.32123538511752886</c:v>
+                  <c:v>0.19768331391847932</c:v>
                 </c:pt>
                 <c:pt idx="79">
-                  <c:v>0.32182852889030422</c:v>
+                  <c:v>0.19804832547095644</c:v>
                 </c:pt>
                 <c:pt idx="80">
-                  <c:v>0.32233978948549169</c:v>
+                  <c:v>0.19836294737568722</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.32277841604000762</c:v>
+                  <c:v>0.19863287140923547</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.32315295543592437</c:v>
+                  <c:v>0.19886335719133807</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.32347125034502283</c:v>
+                  <c:v>0.19905923098155251</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.32374044782105788</c:v>
+                  <c:v>0.19922489096680485</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.32396701697112512</c:v>
+                  <c:v>0.199364318136077</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.32415677421421263</c:v>
+                  <c:v>0.19948109182413087</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.32431491465326501</c:v>
+                  <c:v>0.19957840901739385</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.32444604814158295</c:v>
+                  <c:v>0.19965910654866645</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.3245542387092018</c:v>
+                  <c:v>0.1997256853595088</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.32464304612372757</c:v>
+                  <c:v>0.19978033607614004</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.32471556848661476</c:v>
+                  <c:v>0.19982496522253218</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.32477448490384953</c:v>
+                  <c:v>0.19986122147929203</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.32482209741368234</c:v>
+                  <c:v>0.19989052148534298</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.32486037149823072</c:v>
+                  <c:v>0.19991407476814199</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.3248909746459317</c:v>
+                  <c:v>0.1999329074744195</c:v>
                 </c:pt>
                 <c:pt idx="96">
-                  <c:v>0.32491531256425021</c:v>
+                  <c:v>0.19994788465492319</c:v>
                 </c:pt>
                 <c:pt idx="97">
-                  <c:v>0.32493456276384014</c:v>
+                  <c:v>0.19995973093159392</c:v>
                 </c:pt>
                 <c:pt idx="98">
-                  <c:v>0.32494970534441392</c:v>
+                  <c:v>0.19996904944271626</c:v>
                 </c:pt>
                 <c:pt idx="99">
-                  <c:v>0.32496155090760193</c:v>
+                  <c:v>0.19997633902006273</c:v>
                 </c:pt>
                 <c:pt idx="100">
-                  <c:v>0.32497076560245858</c:v>
+                  <c:v>0.19998200960151297</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1066,6 +1066,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1073,7 +1074,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1327,124 +1327,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.9387164590499728E-6</c:v>
+                  <c:v>1.8084408978769062E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.3508987656584158E-5</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.9336018158404631E-5</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.8802429327882398E-4</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.6713369702505162E-4</c:v>
+                  <c:v>2.2592842893849331E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.3414614007045462E-4</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.006422790718059E-3</c:v>
+                  <c:v>6.1933710198034406E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5011520593627675E-3</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.1352885583158314E-3</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.9254833434584626E-3</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.8880058412656712E-3</c:v>
+                  <c:v>2.3926189792404132E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.0386579732422526E-3</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.3926811083940913E-3</c:v>
+                  <c:v>3.9339576051655948E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>7.9646566013662247E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>9.7684008073131972E-3</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.1816855602081967E-2</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.4121975575197189E-2</c:v>
+                  <c:v>8.6904465078136549E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.6694613200417676E-2</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.9544403420951564E-2</c:v>
+                  <c:v>1.2027325182124038E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.267964921017894E-2</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2.6107209780122643E-2</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.9832393204970647E-2</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.3858855301670994E-2</c:v>
+                  <c:v>2.0836218647182148E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.8188506660006477E-2</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>4.2821429736777793E-2</c:v>
+                  <c:v>2.6351649068786332E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>4.7755807919210802E-2</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.2987868418287974E-2</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.8511840770746393E-2</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>6.4319932607017835E-2</c:v>
+                  <c:v>3.9581496988934053E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.040232418023408E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.6747182948336296E-2</c:v>
+                  <c:v>4.7229035660514646E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8.3340699258080464E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>9.0167143898212704E-2</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>9.7208947972360321E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.10444680519450757</c:v>
+                  <c:v>6.4274957042773889E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.11185979633676199</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.11942553516706651</c:v>
+                  <c:v>7.3492637025887084E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.12712033481123883</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.13491939306780171</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.14279699480482452</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1601,6 +1601,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1608,7 +1609,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1862,124 +1862,124 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.9387164590499728E-6</c:v>
+                  <c:v>1.8084408978769062E-6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.3508987656584158E-5</c:v>
+                  <c:v>1.4467069327128713E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.9336018158404631E-5</c:v>
+                  <c:v>4.8822165020556696E-5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.8802429327882398E-4</c:v>
+                  <c:v>1.1570725740235322E-4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.6713369702505162E-4</c:v>
+                  <c:v>2.2592842893849331E-4</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.3414614007045462E-4</c:v>
+                  <c:v>3.9024377850489512E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.006422790718059E-3</c:v>
+                  <c:v>6.1933710198034406E-4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5011520593627675E-3</c:v>
+                  <c:v>9.2378588268478008E-4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.1352885583158314E-3</c:v>
+                  <c:v>1.314023728194358E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.9254833434584626E-3</c:v>
+                  <c:v>1.8002974421282847E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.8880058412656712E-3</c:v>
+                  <c:v>2.3926189792404132E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>5.0386579732422526E-3</c:v>
+                  <c:v>3.1007125989183093E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>6.3926811083940913E-3</c:v>
+                  <c:v>3.9339576051655948E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>7.9646566013662247E-3</c:v>
+                  <c:v>4.9013271393022924E-3</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>9.7684008073131972E-3</c:v>
+                  <c:v>6.0113235737311978E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.1816855602081967E-2</c:v>
+                  <c:v>7.2719111397427484E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1.4121975575197189E-2</c:v>
+                  <c:v>8.6904465078136549E-3</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.6694613200417676E-2</c:v>
+                  <c:v>1.0273608123333956E-2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.9544403420951564E-2</c:v>
+                  <c:v>1.2027325182124038E-2</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.267964921017894E-2</c:v>
+                  <c:v>1.3956707206263963E-2</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>2.6107209780122643E-2</c:v>
+                  <c:v>1.6065975249306242E-2</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.9832393204970647E-2</c:v>
+                  <c:v>1.8358395818443476E-2</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3.3858855301670994E-2</c:v>
+                  <c:v>2.0836218647182148E-2</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>3.8188506660006477E-2</c:v>
+                  <c:v>2.3500619483080909E-2</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>4.2821429736777793E-2</c:v>
+                  <c:v>2.6351649068786332E-2</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>4.7755807919210802E-2</c:v>
+                  <c:v>2.9388189488745109E-2</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>5.2987868418287974E-2</c:v>
+                  <c:v>3.2607919026638753E-2</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>5.8511840770746393E-2</c:v>
+                  <c:v>3.6007286628151627E-2</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>6.4319932607017835E-2</c:v>
+                  <c:v>3.9581496988934053E-2</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>7.040232418023408E-2</c:v>
+                  <c:v>4.3324507187836363E-2</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>7.6747182948336296E-2</c:v>
+                  <c:v>4.7229035660514646E-2</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>8.3340699258080464E-2</c:v>
+                  <c:v>5.1286584158818753E-2</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>9.0167143898212704E-2</c:v>
+                  <c:v>5.5487473168130901E-2</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>9.7208947972360321E-2</c:v>
+                  <c:v>5.982089105991404E-2</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>0.10444680519450757</c:v>
+                  <c:v>6.4274957042773889E-2</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>0.11185979633676199</c:v>
+                  <c:v>6.8836797745699688E-2</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>0.11942553516706651</c:v>
+                  <c:v>7.3492637025887084E-2</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>0.12712033481123883</c:v>
+                  <c:v>7.8227898345377744E-2</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>0.13491939306780171</c:v>
+                  <c:v>8.3027318810954889E-2</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>0.14279699480482452</c:v>
+                  <c:v>8.787507372604586E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2136,6 +2136,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2143,7 +2144,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4264,33 +4264,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3D2DEE-686E-48A0-AC3D-0F54DEA5D0EC}">
   <dimension ref="A1:C121"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -4298,25 +4298,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>38</v>
       </c>
       <c r="B12">
-        <v>0.32500000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -4324,7 +4324,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -4332,7 +4332,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -4340,7 +4340,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>40</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20">
         <f>(1-EXP(-((C20/$B$16-($B$15-0.5))/$B$13)^$B$14))*$B$12</f>
         <v>0</v>
@@ -4357,1010 +4357,1010 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21">
         <f t="shared" ref="B21:B84" si="0">(1-EXP(-((C21/$B$16-($B$15-0.5))/$B$13)^$B$14))*$B$12</f>
-        <v>2.9387164590499728E-6</v>
+        <v>1.8084408978769062E-6</v>
       </c>
       <c r="C21">
         <f>C20+0.25</f>
         <v>0.25</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22">
         <f t="shared" si="0"/>
-        <v>2.3508987656584158E-5</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="C22">
         <f t="shared" ref="C22:C85" si="1">C21+0.25</f>
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23">
         <f t="shared" si="0"/>
-        <v>7.9336018158404631E-5</v>
+        <v>4.8822165020556696E-5</v>
       </c>
       <c r="C23">
         <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24">
         <f t="shared" si="0"/>
-        <v>1.8802429327882398E-4</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="C24">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25">
         <f t="shared" si="0"/>
-        <v>3.6713369702505162E-4</v>
+        <v>2.2592842893849331E-4</v>
       </c>
       <c r="C25">
         <f t="shared" si="1"/>
         <v>1.25</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26">
         <f t="shared" si="0"/>
-        <v>6.3414614007045462E-4</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="C26">
         <f t="shared" si="1"/>
         <v>1.5</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27">
         <f t="shared" si="0"/>
-        <v>1.006422790718059E-3</v>
+        <v>6.1933710198034406E-4</v>
       </c>
       <c r="C27">
         <f t="shared" si="1"/>
         <v>1.75</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28">
         <f t="shared" si="0"/>
-        <v>1.5011520593627675E-3</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="C28">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29">
         <f t="shared" si="0"/>
-        <v>2.1352885583158314E-3</v>
+        <v>1.314023728194358E-3</v>
       </c>
       <c r="C29">
         <f t="shared" si="1"/>
         <v>2.25</v>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30">
         <f t="shared" si="0"/>
-        <v>2.9254833434584626E-3</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="C30">
         <f t="shared" si="1"/>
         <v>2.5</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31">
         <f t="shared" si="0"/>
-        <v>3.8880058412656712E-3</v>
+        <v>2.3926189792404132E-3</v>
       </c>
       <c r="C31">
         <f t="shared" si="1"/>
         <v>2.75</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B32">
         <f t="shared" si="0"/>
-        <v>5.0386579732422526E-3</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="C32">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33">
         <f t="shared" si="0"/>
-        <v>6.3926811083940913E-3</v>
+        <v>3.9339576051655948E-3</v>
       </c>
       <c r="C33">
         <f t="shared" si="1"/>
         <v>3.25</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34">
         <f t="shared" si="0"/>
-        <v>7.9646566013662247E-3</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="C34">
         <f t="shared" si="1"/>
         <v>3.5</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35">
         <f t="shared" si="0"/>
-        <v>9.7684008073131972E-3</v>
+        <v>6.0113235737311978E-3</v>
       </c>
       <c r="C35">
         <f t="shared" si="1"/>
         <v>3.75</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>1.1816855602081967E-2</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="C36">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>1.4121975575197189E-2</v>
+        <v>8.6904465078136549E-3</v>
       </c>
       <c r="C37">
         <f t="shared" si="1"/>
         <v>4.25</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>1.6694613200417676E-2</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="C38">
         <f t="shared" si="1"/>
         <v>4.5</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>1.9544403420951564E-2</v>
+        <v>1.2027325182124038E-2</v>
       </c>
       <c r="C39">
         <f t="shared" si="1"/>
         <v>4.75</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>2.267964921017894E-2</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="C40">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>2.6107209780122643E-2</v>
+        <v>1.6065975249306242E-2</v>
       </c>
       <c r="C41">
         <f t="shared" si="1"/>
         <v>5.25</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>2.9832393204970647E-2</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="C42">
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>3.3858855301670994E-2</v>
+        <v>2.0836218647182148E-2</v>
       </c>
       <c r="C43">
         <f t="shared" si="1"/>
         <v>5.75</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>3.8188506660006477E-2</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="C44">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>4.2821429736777793E-2</v>
+        <v>2.6351649068786332E-2</v>
       </c>
       <c r="C45">
         <f t="shared" si="1"/>
         <v>6.25</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>4.7755807919210802E-2</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="C46">
         <f t="shared" si="1"/>
         <v>6.5</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>5.2987868418287974E-2</v>
+        <v>3.2607919026638753E-2</v>
       </c>
       <c r="C47">
         <f t="shared" si="1"/>
         <v>6.75</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>5.8511840770746393E-2</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="C48">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>6.4319932607017835E-2</v>
+        <v>3.9581496988934053E-2</v>
       </c>
       <c r="C49">
         <f t="shared" si="1"/>
         <v>7.25</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>7.040232418023408E-2</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="C50">
         <f t="shared" si="1"/>
         <v>7.5</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>7.6747182948336296E-2</v>
+        <v>4.7229035660514646E-2</v>
       </c>
       <c r="C51">
         <f t="shared" si="1"/>
         <v>7.75</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>8.3340699258080464E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="C52">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>9.0167143898212704E-2</v>
+        <v>5.5487473168130901E-2</v>
       </c>
       <c r="C53">
         <f t="shared" si="1"/>
         <v>8.25</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>9.7208947972360321E-2</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="C54">
         <f t="shared" si="1"/>
         <v>8.5</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>0.10444680519450757</v>
+        <v>6.4274957042773889E-2</v>
       </c>
       <c r="C55">
         <f t="shared" si="1"/>
         <v>8.75</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>0.11185979633676199</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="C56">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>0.11942553516706651</v>
+        <v>7.3492637025887084E-2</v>
       </c>
       <c r="C57">
         <f t="shared" si="1"/>
         <v>9.25</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>0.12712033481123883</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="C58">
         <f t="shared" si="1"/>
         <v>9.5</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>0.13491939306780171</v>
+        <v>8.3027318810954889E-2</v>
       </c>
       <c r="C59">
         <f t="shared" si="1"/>
         <v>9.75</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>0.14279699480482452</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="C60">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>0.15072672918526989</v>
+        <v>9.2754910267858384E-2</v>
       </c>
       <c r="C61">
         <f t="shared" si="1"/>
         <v>10.25</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>0.15868171911122922</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="C62">
         <f t="shared" si="1"/>
         <v>10.5</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>0.16663485995800573</v>
+        <v>0.10254452920492661</v>
       </c>
       <c r="C63">
         <f t="shared" si="1"/>
         <v>10.75</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>0.17455906439599175</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="C64">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>0.18242750988073522</v>
+        <v>0.11226308300352937</v>
       </c>
       <c r="C65">
         <f t="shared" si="1"/>
         <v>11.25</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>0.19021388523755758</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="C66">
         <f t="shared" si="1"/>
         <v>11.5</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>0.19789263268329291</v>
+        <v>0.12178008165125719</v>
       </c>
       <c r="C67">
         <f t="shared" si="1"/>
         <v>11.75</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B68">
         <f t="shared" si="0"/>
-        <v>0.20543918161928124</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="C68">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B69">
         <f t="shared" si="0"/>
-        <v>0.21283017059990736</v>
+        <v>0.13097241267686607</v>
       </c>
       <c r="C69">
         <f t="shared" si="1"/>
         <v>12.25</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B70">
         <f t="shared" si="0"/>
-        <v>0.22004365403087262</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="C70">
         <f t="shared" si="1"/>
         <v>12.5</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B71">
         <f t="shared" si="0"/>
-        <v>0.22705929037995962</v>
+        <v>0.13972879407997515</v>
       </c>
       <c r="C71">
         <f t="shared" si="1"/>
         <v>12.75</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B72">
         <f t="shared" si="0"/>
-        <v>0.23385850898689628</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="C72">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B73">
         <f t="shared" si="0"/>
-        <v>0.24042465293238419</v>
+        <v>0.14795363257377489</v>
       </c>
       <c r="C73">
         <f t="shared" si="1"/>
         <v>13.25</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B74">
         <f t="shared" si="0"/>
-        <v>0.2467430958615193</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="C74">
         <f t="shared" si="1"/>
         <v>13.5</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B75">
         <f t="shared" si="0"/>
-        <v>0.25280133114377951</v>
+        <v>0.15557004993463353</v>
       </c>
       <c r="C75">
         <f t="shared" si="1"/>
         <v>13.75</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B76">
         <f t="shared" si="0"/>
-        <v>0.2585890322787715</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="C76">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B77">
         <f t="shared" si="0"/>
-        <v>0.26409808401086282</v>
+        <v>0.16252189785283866</v>
       </c>
       <c r="C77">
         <f t="shared" si="1"/>
         <v>14.25</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B78">
         <f t="shared" si="0"/>
-        <v>0.26932258418246974</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="C78">
         <f t="shared" si="1"/>
         <v>14.5</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B79">
         <f t="shared" si="0"/>
-        <v>0.27425881692032672</v>
+        <v>0.16877465656635493</v>
       </c>
       <c r="C79">
         <f t="shared" si="1"/>
         <v>14.75</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B80">
         <f t="shared" si="0"/>
-        <v>0.2789051982966137</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="C80">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B81">
         <f t="shared" si="0"/>
-        <v>0.28326219612285092</v>
+        <v>0.17431519761406211</v>
       </c>
       <c r="C81">
         <f t="shared" si="1"/>
         <v>15.25</v>
       </c>
     </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B82">
         <f t="shared" si="0"/>
-        <v>0.2873322260053523</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="C82">
         <f t="shared" si="1"/>
         <v>15.5</v>
       </c>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B83">
         <f t="shared" si="0"/>
-        <v>0.29111952620450759</v>
+        <v>0.17915047766431236</v>
       </c>
       <c r="C83">
         <f t="shared" si="1"/>
         <v>15.75</v>
       </c>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B84">
         <f t="shared" si="0"/>
-        <v>0.29463001418577178</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="C84">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B85">
         <f t="shared" ref="B85:B121" si="2">(1-EXP(-((C85/$B$16-($B$15-0.5))/$B$13)^$B$14))*$B$12</f>
-        <v>0.29787112801967686</v>
+        <v>0.18330530955057037</v>
       </c>
       <c r="C85">
         <f t="shared" si="1"/>
         <v>16.25</v>
       </c>
     </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B86">
         <f t="shared" si="2"/>
-        <v>0.30085165597558955</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="C86">
         <f t="shared" ref="C86:C121" si="3">C85+0.25</f>
         <v>16.5</v>
       </c>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B87">
         <f t="shared" si="2"/>
-        <v>0.30358155775609158</v>
+        <v>0.18681942015759484</v>
       </c>
       <c r="C87">
         <f t="shared" si="3"/>
         <v>16.75</v>
       </c>
     </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B88">
         <f t="shared" si="2"/>
-        <v>0.30607178083525383</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="C88">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B89">
         <f t="shared" si="2"/>
-        <v>0.30833407529690587</v>
+        <v>0.18974404633655748</v>
       </c>
       <c r="C89">
         <f t="shared" si="3"/>
         <v>17.25</v>
       </c>
     </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B90">
         <f t="shared" si="2"/>
-        <v>0.31038081042304033</v>
+        <v>0.19100357564494788</v>
       </c>
       <c r="C90">
         <f t="shared" si="3"/>
         <v>17.5</v>
       </c>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B91">
         <f t="shared" si="2"/>
-        <v>0.31222479606484704</v>
+        <v>0.19213833603990588</v>
       </c>
       <c r="C91">
         <f t="shared" si="3"/>
         <v>17.75</v>
       </c>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B92">
         <f t="shared" si="2"/>
-        <v>0.31387911154870857</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="C92">
         <f t="shared" si="3"/>
         <v>18</v>
       </c>
     </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B93">
         <f t="shared" si="2"/>
-        <v>0.31535694453758484</v>
+        <v>0.19406581202312914</v>
       </c>
       <c r="C93">
         <f t="shared" si="3"/>
         <v>18.25</v>
       </c>
     </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B94">
         <f t="shared" si="2"/>
-        <v>0.31667144189658553</v>
+        <v>0.19487473347482187</v>
       </c>
       <c r="C94">
         <f t="shared" si="3"/>
         <v>18.5</v>
       </c>
     </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B95">
         <f t="shared" si="2"/>
-        <v>0.3178355742128724</v>
+        <v>0.19559112259253686</v>
       </c>
       <c r="C95">
         <f t="shared" si="3"/>
         <v>18.75</v>
       </c>
     </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B96">
         <f t="shared" si="2"/>
-        <v>0.31886201520731511</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="C96">
         <f t="shared" si="3"/>
         <v>19</v>
       </c>
     </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B97">
         <f t="shared" si="2"/>
-        <v>0.31976303686122226</v>
+        <v>0.19677725345305985</v>
       </c>
       <c r="C97">
         <f t="shared" si="3"/>
         <v>19.25</v>
       </c>
     </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B98">
         <f t="shared" si="2"/>
-        <v>0.32055042067798994</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="C98">
         <f t="shared" si="3"/>
         <v>19.5</v>
       </c>
     </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B99">
         <f t="shared" si="2"/>
-        <v>0.32123538511752886</v>
+        <v>0.19768331391847932</v>
       </c>
       <c r="C99">
         <f t="shared" si="3"/>
         <v>19.75</v>
       </c>
     </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B100">
         <f t="shared" si="2"/>
-        <v>0.32182852889030422</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="C100">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
     </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B101">
         <f t="shared" si="2"/>
-        <v>0.32233978948549169</v>
+        <v>0.19836294737568722</v>
       </c>
       <c r="C101">
         <f t="shared" si="3"/>
         <v>20.25</v>
       </c>
     </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B102">
         <f t="shared" si="2"/>
-        <v>0.32277841604000762</v>
+        <v>0.19863287140923547</v>
       </c>
       <c r="C102">
         <f t="shared" si="3"/>
         <v>20.5</v>
       </c>
     </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B103">
         <f t="shared" si="2"/>
-        <v>0.32315295543592437</v>
+        <v>0.19886335719133807</v>
       </c>
       <c r="C103">
         <f t="shared" si="3"/>
         <v>20.75</v>
       </c>
     </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B104">
         <f t="shared" si="2"/>
-        <v>0.32347125034502283</v>
+        <v>0.19905923098155251</v>
       </c>
       <c r="C104">
         <f t="shared" si="3"/>
         <v>21</v>
       </c>
     </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B105">
         <f t="shared" si="2"/>
-        <v>0.32374044782105788</v>
+        <v>0.19922489096680485</v>
       </c>
       <c r="C105">
         <f t="shared" si="3"/>
         <v>21.25</v>
       </c>
     </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B106">
         <f t="shared" si="2"/>
-        <v>0.32396701697112512</v>
+        <v>0.199364318136077</v>
       </c>
       <c r="C106">
         <f t="shared" si="3"/>
         <v>21.5</v>
       </c>
     </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B107">
         <f t="shared" si="2"/>
-        <v>0.32415677421421263</v>
+        <v>0.19948109182413087</v>
       </c>
       <c r="C107">
         <f t="shared" si="3"/>
         <v>21.75</v>
       </c>
     </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B108">
         <f t="shared" si="2"/>
-        <v>0.32431491465326501</v>
+        <v>0.19957840901739385</v>
       </c>
       <c r="C108">
         <f t="shared" si="3"/>
         <v>22</v>
       </c>
     </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B109">
         <f t="shared" si="2"/>
-        <v>0.32444604814158295</v>
+        <v>0.19965910654866645</v>
       </c>
       <c r="C109">
         <f t="shared" si="3"/>
         <v>22.25</v>
       </c>
     </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B110">
         <f t="shared" si="2"/>
-        <v>0.3245542387092018</v>
+        <v>0.1997256853595088</v>
       </c>
       <c r="C110">
         <f t="shared" si="3"/>
         <v>22.5</v>
       </c>
     </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B111">
         <f t="shared" si="2"/>
-        <v>0.32464304612372757</v>
+        <v>0.19978033607614004</v>
       </c>
       <c r="C111">
         <f t="shared" si="3"/>
         <v>22.75</v>
       </c>
     </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B112">
         <f t="shared" si="2"/>
-        <v>0.32471556848661476</v>
+        <v>0.19982496522253218</v>
       </c>
       <c r="C112">
         <f t="shared" si="3"/>
         <v>23</v>
       </c>
     </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B113">
         <f t="shared" si="2"/>
-        <v>0.32477448490384953</v>
+        <v>0.19986122147929203</v>
       </c>
       <c r="C113">
         <f t="shared" si="3"/>
         <v>23.25</v>
       </c>
     </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B114">
         <f t="shared" si="2"/>
-        <v>0.32482209741368234</v>
+        <v>0.19989052148534298</v>
       </c>
       <c r="C114">
         <f t="shared" si="3"/>
         <v>23.5</v>
       </c>
     </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B115">
         <f t="shared" si="2"/>
-        <v>0.32486037149823072</v>
+        <v>0.19991407476814199</v>
       </c>
       <c r="C115">
         <f t="shared" si="3"/>
         <v>23.75</v>
       </c>
     </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B116">
         <f t="shared" si="2"/>
-        <v>0.3248909746459317</v>
+        <v>0.1999329074744195</v>
       </c>
       <c r="C116">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
     </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B117">
         <f t="shared" si="2"/>
-        <v>0.32491531256425021</v>
+        <v>0.19994788465492319</v>
       </c>
       <c r="C117">
         <f t="shared" si="3"/>
         <v>24.25</v>
       </c>
     </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B118">
         <f t="shared" si="2"/>
-        <v>0.32493456276384014</v>
+        <v>0.19995973093159392</v>
       </c>
       <c r="C118">
         <f t="shared" si="3"/>
         <v>24.5</v>
       </c>
     </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B119">
         <f t="shared" si="2"/>
-        <v>0.32494970534441392</v>
+        <v>0.19996904944271626</v>
       </c>
       <c r="C119">
         <f t="shared" si="3"/>
         <v>24.75</v>
       </c>
     </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B120">
         <f t="shared" si="2"/>
-        <v>0.32496155090760193</v>
+        <v>0.19997633902006273</v>
       </c>
       <c r="C120">
         <f t="shared" si="3"/>
         <v>25</v>
       </c>
     </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B121">
         <f t="shared" si="2"/>
-        <v>0.32497076560245858</v>
+        <v>0.19998200960151297</v>
       </c>
       <c r="C121">
         <f t="shared" si="3"/>
@@ -5379,13 +5379,13 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:CE2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:83" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:83" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -5395,330 +5395,330 @@
       </c>
       <c r="C1">
         <f>(1-EXP(-((C2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.9387164590499728E-6</v>
+        <v>1.8084408978769062E-6</v>
       </c>
       <c r="D1">
         <f>(1-EXP(-((D2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.3508987656584158E-5</v>
+        <v>1.4467069327128713E-5</v>
       </c>
       <c r="E1">
         <f>(1-EXP(-((E2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>7.9336018158404631E-5</v>
+        <v>4.8822165020556696E-5</v>
       </c>
       <c r="F1">
         <f>(1-EXP(-((F2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.8802429327882398E-4</v>
+        <v>1.1570725740235322E-4</v>
       </c>
       <c r="G1">
         <f>(1-EXP(-((G2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>3.6713369702505162E-4</v>
+        <v>2.2592842893849331E-4</v>
       </c>
       <c r="H1">
         <f>(1-EXP(-((H2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>6.3414614007045462E-4</v>
+        <v>3.9024377850489512E-4</v>
       </c>
       <c r="I1">
         <f>(1-EXP(-((I2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.006422790718059E-3</v>
+        <v>6.1933710198034406E-4</v>
       </c>
       <c r="J1">
         <f>(1-EXP(-((J2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.5011520593627675E-3</v>
+        <v>9.2378588268478008E-4</v>
       </c>
       <c r="K1">
         <f>(1-EXP(-((K2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.1352885583158314E-3</v>
+        <v>1.314023728194358E-3</v>
       </c>
       <c r="L1">
         <f>(1-EXP(-((L2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.9254833434584626E-3</v>
+        <v>1.8002974421282847E-3</v>
       </c>
       <c r="M1">
         <f>(1-EXP(-((M2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>3.8880058412656712E-3</v>
+        <v>2.3926189792404132E-3</v>
       </c>
       <c r="N1">
         <f>(1-EXP(-((N2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>5.0386579732422526E-3</v>
+        <v>3.1007125989183093E-3</v>
       </c>
       <c r="O1">
         <f>(1-EXP(-((O2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>6.3926811083940913E-3</v>
+        <v>3.9339576051655948E-3</v>
       </c>
       <c r="P1">
         <f>(1-EXP(-((P2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>7.9646566013662247E-3</v>
+        <v>4.9013271393022924E-3</v>
       </c>
       <c r="Q1">
         <f>(1-EXP(-((Q2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>9.7684008073131972E-3</v>
+        <v>6.0113235737311978E-3</v>
       </c>
       <c r="R1">
         <f>(1-EXP(-((R2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.1816855602081967E-2</v>
+        <v>7.2719111397427484E-3</v>
       </c>
       <c r="S1">
         <f>(1-EXP(-((S2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.4121975575197189E-2</v>
+        <v>8.6904465078136549E-3</v>
       </c>
       <c r="T1">
         <f>(1-EXP(-((T2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.6694613200417676E-2</v>
+        <v>1.0273608123333956E-2</v>
       </c>
       <c r="U1">
         <f>(1-EXP(-((U2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>1.9544403420951564E-2</v>
+        <v>1.2027325182124038E-2</v>
       </c>
       <c r="V1">
         <f>(1-EXP(-((V2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.267964921017894E-2</v>
+        <v>1.3956707206263963E-2</v>
       </c>
       <c r="W1">
         <f>(1-EXP(-((W2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.6107209780122643E-2</v>
+        <v>1.6065975249306242E-2</v>
       </c>
       <c r="X1">
         <f>(1-EXP(-((X2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>2.9832393204970647E-2</v>
+        <v>1.8358395818443476E-2</v>
       </c>
       <c r="Y1">
         <f>(1-EXP(-((Y2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>3.3858855301670994E-2</v>
+        <v>2.0836218647182148E-2</v>
       </c>
       <c r="Z1">
         <f>(1-EXP(-((Z2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>3.8188506660006477E-2</v>
+        <v>2.3500619483080909E-2</v>
       </c>
       <c r="AA1">
         <f>(1-EXP(-((AA2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>4.2821429736777793E-2</v>
+        <v>2.6351649068786332E-2</v>
       </c>
       <c r="AB1">
         <f>(1-EXP(-((AB2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>4.7755807919210802E-2</v>
+        <v>2.9388189488745109E-2</v>
       </c>
       <c r="AC1">
         <f>(1-EXP(-((AC2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>5.2987868418287974E-2</v>
+        <v>3.2607919026638753E-2</v>
       </c>
       <c r="AD1">
         <f>(1-EXP(-((AD2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>5.8511840770746393E-2</v>
+        <v>3.6007286628151627E-2</v>
       </c>
       <c r="AE1">
         <f>(1-EXP(-((AE2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>6.4319932607017835E-2</v>
+        <v>3.9581496988934053E-2</v>
       </c>
       <c r="AF1">
         <f>(1-EXP(-((AF2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>7.040232418023408E-2</v>
+        <v>4.3324507187836363E-2</v>
       </c>
       <c r="AG1">
         <f>(1-EXP(-((AG2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>7.6747182948336296E-2</v>
+        <v>4.7229035660514646E-2</v>
       </c>
       <c r="AH1">
         <f>(1-EXP(-((AH2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>8.3340699258080464E-2</v>
+        <v>5.1286584158818753E-2</v>
       </c>
       <c r="AI1">
         <f>(1-EXP(-((AI2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>9.0167143898212704E-2</v>
+        <v>5.5487473168130901E-2</v>
       </c>
       <c r="AJ1">
         <f>(1-EXP(-((AJ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>9.7208947972360321E-2</v>
+        <v>5.982089105991404E-2</v>
       </c>
       <c r="AK1">
         <f>(1-EXP(-((AK2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.10444680519450757</v>
+        <v>6.4274957042773889E-2</v>
       </c>
       <c r="AL1">
         <f>(1-EXP(-((AL2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.11185979633676199</v>
+        <v>6.8836797745699688E-2</v>
       </c>
       <c r="AM1">
         <f>(1-EXP(-((AM2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.11942553516706651</v>
+        <v>7.3492637025887084E-2</v>
       </c>
       <c r="AN1">
         <f>(1-EXP(-((AN2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.12712033481123883</v>
+        <v>7.8227898345377744E-2</v>
       </c>
       <c r="AO1">
         <f>(1-EXP(-((AO2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.13491939306780171</v>
+        <v>8.3027318810954889E-2</v>
       </c>
       <c r="AP1">
         <f>(1-EXP(-((AP2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.14279699480482452</v>
+        <v>8.787507372604586E-2</v>
       </c>
       <c r="AQ1">
         <f>(1-EXP(-((AQ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.15072672918526989</v>
+        <v>9.2754910267858384E-2</v>
       </c>
       <c r="AR1">
         <f>(1-EXP(-((AR2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.15868171911122922</v>
+        <v>9.7650288683833367E-2</v>
       </c>
       <c r="AS1">
         <f>(1-EXP(-((AS2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.16663485995800573</v>
+        <v>0.10254452920492661</v>
       </c>
       <c r="AT1">
         <f>(1-EXP(-((AT2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.17455906439599175</v>
+        <v>0.10742096270522571</v>
       </c>
       <c r="AU1">
         <f>(1-EXP(-((AU2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.18242750988073522</v>
+        <v>0.11226308300352937</v>
       </c>
       <c r="AV1">
         <f>(1-EXP(-((AV2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.19021388523755758</v>
+        <v>0.11705469860772776</v>
       </c>
       <c r="AW1">
         <f>(1-EXP(-((AW2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.19789263268329291</v>
+        <v>0.12178008165125719</v>
       </c>
       <c r="AX1">
         <f>(1-EXP(-((AX2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.20543918161928124</v>
+        <v>0.12642411176571153</v>
       </c>
       <c r="AY1">
         <f>(1-EXP(-((AY2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.21283017059990736</v>
+        <v>0.13097241267686607</v>
       </c>
       <c r="AZ1">
         <f>(1-EXP(-((AZ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.22004365403087262</v>
+        <v>0.13541147940361392</v>
       </c>
       <c r="BA1">
         <f>(1-EXP(-((BA2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.22705929037995962</v>
+        <v>0.13972879407997515</v>
       </c>
       <c r="BB1">
         <f>(1-EXP(-((BB2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.23385850898689628</v>
+        <v>0.1439129286073208</v>
       </c>
       <c r="BC1">
         <f>(1-EXP(-((BC2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.24042465293238419</v>
+        <v>0.14795363257377489</v>
       </c>
       <c r="BD1">
         <f>(1-EXP(-((BD2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.2467430958615193</v>
+        <v>0.15184190514555035</v>
       </c>
       <c r="BE1">
         <f>(1-EXP(-((BE2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.25280133114377951</v>
+        <v>0.15557004993463353</v>
       </c>
       <c r="BF1">
         <f>(1-EXP(-((BF2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.2585890322787715</v>
+        <v>0.1591317121715517</v>
       </c>
       <c r="BG1">
         <f>(1-EXP(-((BG2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.26409808401086282</v>
+        <v>0.16252189785283866</v>
       </c>
       <c r="BH1">
         <f>(1-EXP(-((BH2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.26932258418246974</v>
+        <v>0.16573697488151984</v>
       </c>
       <c r="BI1">
         <f>(1-EXP(-((BI2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.27425881692032672</v>
+        <v>0.16877465656635493</v>
       </c>
       <c r="BJ1">
         <f>(1-EXP(-((BJ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.2789051982966137</v>
+        <v>0.17163396818253152</v>
       </c>
       <c r="BK1">
         <f>(1-EXP(-((BK2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.28326219612285092</v>
+        <v>0.17431519761406211</v>
       </c>
       <c r="BL1">
         <f>(1-EXP(-((BL2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.2873322260053523</v>
+        <v>0.17681983138790913</v>
       </c>
       <c r="BM1">
         <f>(1-EXP(-((BM2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.29111952620450759</v>
+        <v>0.17915047766431236</v>
       </c>
       <c r="BN1">
         <f>(1-EXP(-((BN2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.29463001418577178</v>
+        <v>0.18131077796047496</v>
       </c>
       <c r="BO1">
         <f>(1-EXP(-((BO2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.29787112801967686</v>
+        <v>0.18330530955057037</v>
       </c>
       <c r="BP1">
         <f>(1-EXP(-((BP2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.30085165597558955</v>
+        <v>0.18513948060036278</v>
       </c>
       <c r="BQ1">
         <f>(1-EXP(-((BQ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.30358155775609158</v>
+        <v>0.18681942015759484</v>
       </c>
       <c r="BR1">
         <f>(1-EXP(-((BR2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.30607178083525383</v>
+        <v>0.18835186512938695</v>
       </c>
       <c r="BS1">
         <f>(1-EXP(-((BS2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.30833407529690587</v>
+        <v>0.18974404633655748</v>
       </c>
       <c r="BT1">
         <f>(1-EXP(-((BT2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31038081042304033</v>
+        <v>0.19100357564494788</v>
       </c>
       <c r="BU1">
         <f>(1-EXP(-((BU2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31222479606484704</v>
+        <v>0.19213833603990588</v>
       </c>
       <c r="BV1">
         <f>(1-EXP(-((BV2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31387911154870857</v>
+        <v>0.1931563763376668</v>
       </c>
       <c r="BW1">
         <f>(1-EXP(-((BW2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31535694453758484</v>
+        <v>0.19406581202312914</v>
       </c>
       <c r="BX1">
         <f>(1-EXP(-((BX2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31667144189658553</v>
+        <v>0.19487473347482187</v>
       </c>
       <c r="BY1">
         <f>(1-EXP(-((BY2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.3178355742128724</v>
+        <v>0.19559112259253686</v>
       </c>
       <c r="BZ1">
         <f>(1-EXP(-((BZ2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31886201520731511</v>
+        <v>0.19622277858911699</v>
       </c>
       <c r="CA1">
         <f>(1-EXP(-((CA2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.31976303686122226</v>
+        <v>0.19677725345305985</v>
       </c>
       <c r="CB1">
         <f>(1-EXP(-((CB2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.32055042067798994</v>
+        <v>0.1972617973403015</v>
       </c>
       <c r="CC1">
         <f>(1-EXP(-((CC2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.32123538511752886</v>
+        <v>0.19768331391847932</v>
       </c>
       <c r="CD1">
         <f>(1-EXP(-((CD2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.32182852889030422</v>
+        <v>0.19804832547095644</v>
       </c>
       <c r="CE1">
         <f>(1-EXP(-((CE2/About!$B$16-(About!$B$15-0.5))/About!$B$13)^About!$B$14))*About!$B$12</f>
-        <v>0.32500000000000001</v>
-      </c>
-    </row>
-    <row r="2" spans="1:83" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:83" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -6061,17 +6061,17 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>35</v>
       </c>
@@ -6090,12 +6090,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -6285,7 +6285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6380,7 +6380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6570,7 +6570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -6665,7 +6665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -6760,7 +6760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6855,7 +6855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -7045,7 +7045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -7140,7 +7140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -7235,7 +7235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -7330,7 +7330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -7425,7 +7425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -7520,7 +7520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -7615,7 +7615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -7710,7 +7710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -7805,7 +7805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -7900,7 +7900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -7995,7 +7995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -8090,7 +8090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -8185,7 +8185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -8280,7 +8280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8375,7 +8375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -8476,6 +8476,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -8619,29 +8634,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BEA6468-0943-47D7-A588-67FBB8F1B3FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B605649-CF77-46FD-9B3F-D11F1F265A70}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CC71EE6-D8B3-4D79-A65E-99E7313EF7B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CC71EE6-D8B3-4D79-A65E-99E7313EF7B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B605649-CF77-46FD-9B3F-D11F1F265A70}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BEA6468-0943-47D7-A588-67FBB8F1B3FD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>